<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@46d26ebfb62358059db67f37613672a78b9d8e2b 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Organization.xlsx
+++ b/StructureDefinition-Organization.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-08-19T08:48:07+00:00</t>
+    <t>2024-08-20T13:49:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -297,7 +297,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-1:If the resource is contained in another resource, it SHALL NOT contain any narrative {contained.text.empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource {contained.where(('#'+id in %resource.descendants().reference).not()).empty()}org-1:The organization SHALL at least have a name or an id, and possibly more than one {(identifier.count() + name.count()) &gt; 0}zv-org-1:Organization AGB SHALL be present. {identifier.where(system='http://fhir.nl/fhir/NamingSystem/agb-z') or identifier.where(system='urn:oid:2.16.840.1.113883.2.4.6.1')}</t>
+dom-1:If the resource is contained in another resource, it SHALL NOT contain any narrative {contained.text.empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource {contained.where(('#'+id in %resource.descendants().reference).not()).empty()}org-1:The organization SHALL at least have a name or an id, and possibly more than one {(identifier.count() + name.count()) &gt; 0}zv-org-1:Organization AGB SHALL be present. {identifier.where(system='http://fhir.nl/fhir/NamingSystem/agb-z')}</t>
   </si>
   <si>
     <t>NL-CM:17.2.1</t>
@@ -3628,7 +3628,7 @@
         <v>87</v>
       </c>
       <c r="H12" t="s" s="2">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="I12" t="s" s="2">
         <v>88</v>

</xml_diff>